<commit_message>
Prospection : analyse de la liste Vibe (50 entreprises alimentaires), 5 joignables ajoutées en vague 4 au fichier de suivi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RavxZb3XR9FuiiE8cVSRNP
</commit_message>
<xml_diff>
--- a/produits/templates-entreprises/prospection-stock/prospection_50_entreprises.xlsx
+++ b/produits/templates-entreprises/prospection-stock/prospection_50_entreprises.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Messages" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Prospects!$A$4:$P$51</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Prospects!$A$4:$P$56</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="204">
   <si>
     <t xml:space="preserve">Suivi de la prospection</t>
   </si>
@@ -45,6 +45,9 @@
     <t xml:space="preserve">Vague 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Vague 4</t>
+  </si>
+  <si>
     <t xml:space="preserve">À contacter</t>
   </si>
   <si>
@@ -532,6 +535,75 @@
   </si>
   <si>
     <t xml:space="preserve">Traitement d'eau</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUTAMU ASPK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bukavu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+243 997 374 225</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Farines de bouillie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alimentaire et boissons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liste Vibe. WhatsApp trouvé sur ButamuCare (leur appli de nutrition) : vérifier que c'est la même équipe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UMANDE FOODS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+260 970 463 609</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Légumes déshydratés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liste Vibe. Numéro zambien (+260) trouvé sur leur site, e-mail umandesarl@gmail.com : écrire plutôt par e-mail ou vérifier le WhatsApp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIOFOODS CONGO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+243 895 895 888</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Livraison produits alimentaires (poissons, viandes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liste Vibe. WhatsApp de Mme Lisette (Sales Manager) donné dans leur description. Aussi : appel +243 81 222 9100, biofoodscongo@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIDEMA (MINOTERIE DE MATADI)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+243 81 555 8000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minoterie (farines, aliments bétail)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liste Vibe. Standard de l'entreprise (51 à 200 employés) : demander le responsable commercial ou logistique. Peut-être déjà équipée d'un logiciel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRIGOCONGO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+243 997 022 378</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau de boucheries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liste Vibe. Numéro trouvé sur leur page Facebook (info@frigocongo.com). Vérifier que c'est bien un WhatsApp</t>
   </si>
   <si>
     <t xml:space="preserve">Les messages (vous)</t>
@@ -557,7 +629,8 @@
 • Habillement : Entre les modèles, les tailles et les couleurs, savoir tout de suite si un article est encore disponible n'est pas toujours simple.
 • Entrepôt et distribution : Quand la marchandise entre et sort tous les jours, garder un stock juste et savoir quoi recommander devient vite un travail à plein temps.
 • Pharmacie : Avec autant de références, une rupture passe vite inaperçue, et un client qui ne trouve pas son produit va ailleurs.
-• À vérifier : Quand la marchandise entre et sort tous les jours, garder un stock juste prend vite du temps.</t>
+• À vérifier : Quand la marchandise entre et sort tous les jours, garder un stock juste prend vite du temps.
+• Alimentaire et boissons : Entre la production, les arrivages et les livraisons, savoir ce qu'il reste de chaque produit prend vite du temps.</t>
   </si>
   <si>
     <t xml:space="preserve">Message 2 (s'il répond) + vidéo du workflow</t>
@@ -1232,7 +1305,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:F23"/>
+  <dimension ref="B1:G23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1261,214 +1334,257 @@
       <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="G3" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" s="3" t="n">
-        <f aca="false">COUNTIF(Prospects!$K$5:$K$51,B4)</f>
-        <v>47</v>
+        <f aca="false">COUNTIF(Prospects!$K$5:$K$56,B4)</f>
+        <v>52</v>
       </c>
       <c r="D4" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B4,Prospects!$B$5:$B$51,1)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B4,Prospects!$B$5:$B$56,1)</f>
         <v>20</v>
       </c>
       <c r="E4" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B4,Prospects!$B$5:$B$51,2)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B4,Prospects!$B$5:$B$56,2)</f>
         <v>16</v>
       </c>
       <c r="F4" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B4,Prospects!$B$5:$B$51,3)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B4,Prospects!$B$5:$B$56,3)</f>
         <v>11</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B4,Prospects!$B$5:$B$56,4)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5" s="3" t="n">
-        <f aca="false">COUNTIF(Prospects!$K$5:$K$51,B5)</f>
+        <f aca="false">COUNTIF(Prospects!$K$5:$K$56,B5)</f>
         <v>0</v>
       </c>
       <c r="D5" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B5,Prospects!$B$5:$B$51,1)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B5,Prospects!$B$5:$B$56,1)</f>
         <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B5,Prospects!$B$5:$B$51,2)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B5,Prospects!$B$5:$B$56,2)</f>
         <v>0</v>
       </c>
       <c r="F5" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B5,Prospects!$B$5:$B$51,3)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B5,Prospects!$B$5:$B$56,3)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B5,Prospects!$B$5:$B$56,4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C6" s="3" t="n">
-        <f aca="false">COUNTIF(Prospects!$K$5:$K$51,B6)</f>
+        <f aca="false">COUNTIF(Prospects!$K$5:$K$56,B6)</f>
         <v>0</v>
       </c>
       <c r="D6" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B6,Prospects!$B$5:$B$51,1)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B6,Prospects!$B$5:$B$56,1)</f>
         <v>0</v>
       </c>
       <c r="E6" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B6,Prospects!$B$5:$B$51,2)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B6,Prospects!$B$5:$B$56,2)</f>
         <v>0</v>
       </c>
       <c r="F6" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B6,Prospects!$B$5:$B$51,3)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B6,Prospects!$B$5:$B$56,3)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B6,Prospects!$B$5:$B$56,4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C7" s="3" t="n">
-        <f aca="false">COUNTIF(Prospects!$K$5:$K$51,B7)</f>
+        <f aca="false">COUNTIF(Prospects!$K$5:$K$56,B7)</f>
         <v>0</v>
       </c>
       <c r="D7" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B7,Prospects!$B$5:$B$51,1)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B7,Prospects!$B$5:$B$56,1)</f>
         <v>0</v>
       </c>
       <c r="E7" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B7,Prospects!$B$5:$B$51,2)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B7,Prospects!$B$5:$B$56,2)</f>
         <v>0</v>
       </c>
       <c r="F7" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B7,Prospects!$B$5:$B$51,3)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B7,Prospects!$B$5:$B$56,3)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B7,Prospects!$B$5:$B$56,4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3" t="n">
-        <f aca="false">COUNTIF(Prospects!$K$5:$K$51,B8)</f>
+        <f aca="false">COUNTIF(Prospects!$K$5:$K$56,B8)</f>
         <v>0</v>
       </c>
       <c r="D8" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B8,Prospects!$B$5:$B$51,1)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B8,Prospects!$B$5:$B$56,1)</f>
         <v>0</v>
       </c>
       <c r="E8" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B8,Prospects!$B$5:$B$51,2)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B8,Prospects!$B$5:$B$56,2)</f>
         <v>0</v>
       </c>
       <c r="F8" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B8,Prospects!$B$5:$B$51,3)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B8,Prospects!$B$5:$B$56,3)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B8,Prospects!$B$5:$B$56,4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" s="3" t="n">
-        <f aca="false">COUNTIF(Prospects!$K$5:$K$51,B9)</f>
+        <f aca="false">COUNTIF(Prospects!$K$5:$K$56,B9)</f>
         <v>0</v>
       </c>
       <c r="D9" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B9,Prospects!$B$5:$B$51,1)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B9,Prospects!$B$5:$B$56,1)</f>
         <v>0</v>
       </c>
       <c r="E9" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B9,Prospects!$B$5:$B$51,2)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B9,Prospects!$B$5:$B$56,2)</f>
         <v>0</v>
       </c>
       <c r="F9" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B9,Prospects!$B$5:$B$51,3)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B9,Prospects!$B$5:$B$56,3)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B9,Prospects!$B$5:$B$56,4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C10" s="3" t="n">
-        <f aca="false">COUNTIF(Prospects!$K$5:$K$51,B10)</f>
+        <f aca="false">COUNTIF(Prospects!$K$5:$K$56,B10)</f>
         <v>0</v>
       </c>
       <c r="D10" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B10,Prospects!$B$5:$B$51,1)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B10,Prospects!$B$5:$B$56,1)</f>
         <v>0</v>
       </c>
       <c r="E10" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B10,Prospects!$B$5:$B$51,2)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B10,Prospects!$B$5:$B$56,2)</f>
         <v>0</v>
       </c>
       <c r="F10" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B10,Prospects!$B$5:$B$51,3)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B10,Prospects!$B$5:$B$56,3)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B10,Prospects!$B$5:$B$56,4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" s="3" t="n">
-        <f aca="false">COUNTIF(Prospects!$K$5:$K$51,B11)</f>
+        <f aca="false">COUNTIF(Prospects!$K$5:$K$56,B11)</f>
         <v>0</v>
       </c>
       <c r="D11" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B11,Prospects!$B$5:$B$51,1)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B11,Prospects!$B$5:$B$56,1)</f>
         <v>0</v>
       </c>
       <c r="E11" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B11,Prospects!$B$5:$B$51,2)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B11,Prospects!$B$5:$B$56,2)</f>
         <v>0</v>
       </c>
       <c r="F11" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B11,Prospects!$B$5:$B$51,3)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B11,Prospects!$B$5:$B$56,3)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B11,Prospects!$B$5:$B$56,4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C12" s="3" t="n">
-        <f aca="false">COUNTIF(Prospects!$K$5:$K$51,B12)</f>
+        <f aca="false">COUNTIF(Prospects!$K$5:$K$56,B12)</f>
         <v>0</v>
       </c>
       <c r="D12" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B12,Prospects!$B$5:$B$51,1)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B12,Prospects!$B$5:$B$56,1)</f>
         <v>0</v>
       </c>
       <c r="E12" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B12,Prospects!$B$5:$B$51,2)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B12,Prospects!$B$5:$B$56,2)</f>
         <v>0</v>
       </c>
       <c r="F12" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B12,Prospects!$B$5:$B$51,3)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B12,Prospects!$B$5:$B$56,3)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B12,Prospects!$B$5:$B$56,4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C13" s="3" t="n">
-        <f aca="false">COUNTIF(Prospects!$K$5:$K$51,B13)</f>
+        <f aca="false">COUNTIF(Prospects!$K$5:$K$56,B13)</f>
         <v>0</v>
       </c>
       <c r="D13" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B13,Prospects!$B$5:$B$51,1)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B13,Prospects!$B$5:$B$56,1)</f>
         <v>0</v>
       </c>
       <c r="E13" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B13,Prospects!$B$5:$B$51,2)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B13,Prospects!$B$5:$B$56,2)</f>
         <v>0</v>
       </c>
       <c r="F13" s="3" t="n">
-        <f aca="false">COUNTIFS(Prospects!$K$5:$K$51,$B13,Prospects!$B$5:$B$51,3)</f>
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B13,Prospects!$B$5:$B$56,3)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <f aca="false">COUNTIFS(Prospects!$K$5:$K$56,$B13,Prospects!$B$5:$B$56,4)</f>
         <v>0</v>
       </c>
     </row>
@@ -1478,17 +1594,17 @@
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">SUM(C4:C13)</f>
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C17" s="6" t="n">
         <f aca="false">C14-C4</f>
@@ -1497,7 +1613,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C18" s="6" t="n">
         <f aca="false">C8+C9+C10+C11</f>
@@ -1506,7 +1622,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C19" s="7" t="str">
         <f aca="false">IF(C17=0,"-",C18/C17)</f>
@@ -1515,7 +1631,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C20" s="6" t="n">
         <f aca="false">C10+C11</f>
@@ -1524,7 +1640,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C21" s="6" t="n">
         <f aca="false">C11</f>
@@ -1533,7 +1649,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1552,7 +1668,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P51"/>
+  <dimension ref="A1:P56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1574,62 +1690,62 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K4" s="11" t="s">
         <v>1</v>
       </c>
       <c r="L4" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N4" s="11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="O4" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P4" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1640,29 +1756,29 @@
         <v>1</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J5" s="15"/>
       <c r="K5" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L5" s="17" t="str">
         <f aca="false">IF(J5="","",J5+3)</f>
@@ -1687,29 +1803,29 @@
         <v>1</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D6" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="I6" s="13" t="s">
         <v>47</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>46</v>
       </c>
       <c r="J6" s="15"/>
       <c r="K6" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L6" s="17" t="str">
         <f aca="false">IF(J6="","",J6+3)</f>
@@ -1725,7 +1841,7 @@
       </c>
       <c r="O6" s="19"/>
       <c r="P6" s="20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1736,29 +1852,29 @@
         <v>1</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J7" s="15"/>
       <c r="K7" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L7" s="17" t="str">
         <f aca="false">IF(J7="","",J7+3)</f>
@@ -1783,29 +1899,29 @@
         <v>1</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J8" s="15"/>
       <c r="K8" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L8" s="17" t="str">
         <f aca="false">IF(J8="","",J8+3)</f>
@@ -1821,7 +1937,7 @@
       </c>
       <c r="O8" s="19"/>
       <c r="P8" s="20" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1832,29 +1948,29 @@
         <v>1</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J9" s="15"/>
       <c r="K9" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L9" s="17" t="str">
         <f aca="false">IF(J9="","",J9+3)</f>
@@ -1879,29 +1995,29 @@
         <v>1</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J10" s="15"/>
       <c r="K10" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L10" s="17" t="str">
         <f aca="false">IF(J10="","",J10+3)</f>
@@ -1926,29 +2042,29 @@
         <v>1</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J11" s="15"/>
       <c r="K11" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L11" s="17" t="str">
         <f aca="false">IF(J11="","",J11+3)</f>
@@ -1973,29 +2089,29 @@
         <v>1</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J12" s="15"/>
       <c r="K12" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L12" s="17" t="str">
         <f aca="false">IF(J12="","",J12+3)</f>
@@ -2020,29 +2136,29 @@
         <v>1</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J13" s="15"/>
       <c r="K13" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L13" s="17" t="str">
         <f aca="false">IF(J13="","",J13+3)</f>
@@ -2067,29 +2183,29 @@
         <v>1</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J14" s="15"/>
       <c r="K14" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L14" s="17" t="str">
         <f aca="false">IF(J14="","",J14+3)</f>
@@ -2114,29 +2230,29 @@
         <v>1</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J15" s="15"/>
       <c r="K15" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L15" s="17" t="str">
         <f aca="false">IF(J15="","",J15+3)</f>
@@ -2161,29 +2277,29 @@
         <v>1</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J16" s="15"/>
       <c r="K16" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L16" s="17" t="str">
         <f aca="false">IF(J16="","",J16+3)</f>
@@ -2208,29 +2324,29 @@
         <v>1</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G17" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J17" s="15"/>
       <c r="K17" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L17" s="17" t="str">
         <f aca="false">IF(J17="","",J17+3)</f>
@@ -2255,29 +2371,29 @@
         <v>1</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J18" s="15"/>
       <c r="K18" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L18" s="17" t="str">
         <f aca="false">IF(J18="","",J18+3)</f>
@@ -2302,29 +2418,29 @@
         <v>1</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J19" s="15"/>
       <c r="K19" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L19" s="17" t="str">
         <f aca="false">IF(J19="","",J19+3)</f>
@@ -2349,29 +2465,29 @@
         <v>1</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J20" s="15"/>
       <c r="K20" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L20" s="17" t="str">
         <f aca="false">IF(J20="","",J20+3)</f>
@@ -2396,29 +2512,29 @@
         <v>1</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J21" s="15"/>
       <c r="K21" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L21" s="17" t="str">
         <f aca="false">IF(J21="","",J21+3)</f>
@@ -2443,29 +2559,29 @@
         <v>1</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I22" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J22" s="15"/>
       <c r="K22" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L22" s="17" t="str">
         <f aca="false">IF(J22="","",J22+3)</f>
@@ -2490,29 +2606,29 @@
         <v>1</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I23" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J23" s="15"/>
       <c r="K23" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L23" s="17" t="str">
         <f aca="false">IF(J23="","",J23+3)</f>
@@ -2537,29 +2653,29 @@
         <v>1</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J24" s="15"/>
       <c r="K24" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L24" s="17" t="str">
         <f aca="false">IF(J24="","",J24+3)</f>
@@ -2584,29 +2700,29 @@
         <v>2</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I25" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J25" s="15"/>
       <c r="K25" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L25" s="17" t="str">
         <f aca="false">IF(J25="","",J25+3)</f>
@@ -2631,29 +2747,29 @@
         <v>2</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D26" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="G26" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="I26" s="13" t="s">
         <v>95</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="G26" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H26" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="I26" s="13" t="s">
-        <v>94</v>
       </c>
       <c r="J26" s="15"/>
       <c r="K26" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L26" s="17" t="str">
         <f aca="false">IF(J26="","",J26+3)</f>
@@ -2678,29 +2794,29 @@
         <v>2</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I27" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J27" s="15"/>
       <c r="K27" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L27" s="17" t="str">
         <f aca="false">IF(J27="","",J27+3)</f>
@@ -2725,29 +2841,29 @@
         <v>2</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I28" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J28" s="15"/>
       <c r="K28" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L28" s="17" t="str">
         <f aca="false">IF(J28="","",J28+3)</f>
@@ -2772,29 +2888,29 @@
         <v>2</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I29" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J29" s="15"/>
       <c r="K29" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L29" s="17" t="str">
         <f aca="false">IF(J29="","",J29+3)</f>
@@ -2819,29 +2935,29 @@
         <v>2</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I30" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J30" s="15"/>
       <c r="K30" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L30" s="17" t="str">
         <f aca="false">IF(J30="","",J30+3)</f>
@@ -2866,29 +2982,29 @@
         <v>2</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G31" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I31" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J31" s="15"/>
       <c r="K31" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L31" s="17" t="str">
         <f aca="false">IF(J31="","",J31+3)</f>
@@ -2904,7 +3020,7 @@
       </c>
       <c r="O31" s="19"/>
       <c r="P31" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2915,29 +3031,29 @@
         <v>2</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I32" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J32" s="15"/>
       <c r="K32" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L32" s="17" t="str">
         <f aca="false">IF(J32="","",J32+3)</f>
@@ -2962,29 +3078,29 @@
         <v>2</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I33" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J33" s="15"/>
       <c r="K33" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L33" s="17" t="str">
         <f aca="false">IF(J33="","",J33+3)</f>
@@ -3009,29 +3125,29 @@
         <v>2</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I34" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J34" s="15"/>
       <c r="K34" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L34" s="17" t="str">
         <f aca="false">IF(J34="","",J34+3)</f>
@@ -3056,29 +3172,29 @@
         <v>2</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G35" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I35" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J35" s="15"/>
       <c r="K35" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L35" s="17" t="str">
         <f aca="false">IF(J35="","",J35+3)</f>
@@ -3103,29 +3219,29 @@
         <v>2</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I36" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J36" s="15"/>
       <c r="K36" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L36" s="17" t="str">
         <f aca="false">IF(J36="","",J36+3)</f>
@@ -3150,29 +3266,29 @@
         <v>2</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D37" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="E37" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="F37" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="G37" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H37" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="I37" s="13" t="s">
         <v>121</v>
-      </c>
-      <c r="E37" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="F37" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="G37" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H37" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="I37" s="13" t="s">
-        <v>120</v>
       </c>
       <c r="J37" s="15"/>
       <c r="K37" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L37" s="17" t="str">
         <f aca="false">IF(J37="","",J37+3)</f>
@@ -3197,29 +3313,29 @@
         <v>2</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D38" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="E38" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="G38" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H38" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="E38" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="F38" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="G38" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H38" s="13" t="s">
-        <v>123</v>
-      </c>
       <c r="I38" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J38" s="15"/>
       <c r="K38" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L38" s="17" t="str">
         <f aca="false">IF(J38="","",J38+3)</f>
@@ -3244,29 +3360,29 @@
         <v>2</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F39" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I39" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J39" s="15"/>
       <c r="K39" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L39" s="17" t="str">
         <f aca="false">IF(J39="","",J39+3)</f>
@@ -3291,29 +3407,29 @@
         <v>2</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F40" s="13" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I40" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J40" s="15"/>
       <c r="K40" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L40" s="17" t="str">
         <f aca="false">IF(J40="","",J40+3)</f>
@@ -3338,29 +3454,29 @@
         <v>3</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I41" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J41" s="15"/>
       <c r="K41" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L41" s="17" t="str">
         <f aca="false">IF(J41="","",J41+3)</f>
@@ -3376,7 +3492,7 @@
       </c>
       <c r="O41" s="19"/>
       <c r="P41" s="20" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3387,29 +3503,29 @@
         <v>3</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I42" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J42" s="15"/>
       <c r="K42" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L42" s="17" t="str">
         <f aca="false">IF(J42="","",J42+3)</f>
@@ -3434,29 +3550,29 @@
         <v>3</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D43" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="E43" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F43" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="G43" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H43" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="E43" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="F43" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="G43" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H43" s="13" t="s">
-        <v>139</v>
-      </c>
       <c r="I43" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J43" s="15"/>
       <c r="K43" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L43" s="17" t="str">
         <f aca="false">IF(J43="","",J43+3)</f>
@@ -3481,29 +3597,29 @@
         <v>3</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F44" s="13" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H44" s="13" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I44" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J44" s="15"/>
       <c r="K44" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L44" s="17" t="str">
         <f aca="false">IF(J44="","",J44+3)</f>
@@ -3528,29 +3644,29 @@
         <v>3</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H45" s="13" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I45" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J45" s="15"/>
       <c r="K45" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L45" s="17" t="str">
         <f aca="false">IF(J45="","",J45+3)</f>
@@ -3575,29 +3691,29 @@
         <v>3</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F46" s="13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H46" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I46" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J46" s="15"/>
       <c r="K46" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L46" s="17" t="str">
         <f aca="false">IF(J46="","",J46+3)</f>
@@ -3622,29 +3738,29 @@
         <v>3</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D47" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="E47" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="F47" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="G47" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H47" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="I47" s="13" t="s">
         <v>152</v>
-      </c>
-      <c r="E47" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="F47" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="G47" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H47" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="I47" s="13" t="s">
-        <v>151</v>
       </c>
       <c r="J47" s="15"/>
       <c r="K47" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L47" s="17" t="str">
         <f aca="false">IF(J47="","",J47+3)</f>
@@ -3669,29 +3785,29 @@
         <v>3</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F48" s="13" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H48" s="13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I48" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J48" s="15"/>
       <c r="K48" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L48" s="17" t="str">
         <f aca="false">IF(J48="","",J48+3)</f>
@@ -3707,7 +3823,7 @@
       </c>
       <c r="O48" s="19"/>
       <c r="P48" s="20" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3718,29 +3834,29 @@
         <v>3</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H49" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I49" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J49" s="15"/>
       <c r="K49" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L49" s="17" t="str">
         <f aca="false">IF(J49="","",J49+3)</f>
@@ -3756,7 +3872,7 @@
       </c>
       <c r="O49" s="19"/>
       <c r="P49" s="20" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3767,29 +3883,29 @@
         <v>3</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F50" s="13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H50" s="13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I50" s="13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J50" s="15"/>
       <c r="K50" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L50" s="17" t="str">
         <f aca="false">IF(J50="","",J50+3)</f>
@@ -3805,7 +3921,7 @@
       </c>
       <c r="O50" s="19"/>
       <c r="P50" s="20" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3816,29 +3932,29 @@
         <v>3</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F51" s="13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H51" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I51" s="13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J51" s="15"/>
       <c r="K51" s="16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L51" s="17" t="str">
         <f aca="false">IF(J51="","",J51+3)</f>
@@ -3854,12 +3970,257 @@
       </c>
       <c r="O51" s="19"/>
       <c r="P51" s="20" t="s">
-        <v>165</v>
+        <v>166</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="12" t="n">
+        <v>104</v>
+      </c>
+      <c r="B52" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C52" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D52" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="E52" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="F52" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="G52" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H52" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="I52" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="J52" s="15"/>
+      <c r="K52" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="L52" s="17" t="str">
+        <f aca="false">IF(J52="","",J52+3)</f>
+        <v/>
+      </c>
+      <c r="M52" s="17" t="str">
+        <f aca="false">IF(J52="","",J52+7)</f>
+        <v/>
+      </c>
+      <c r="N52" s="18" t="str">
+        <f aca="true">IF(K52="À contacter","Envoyer message 1 + vidéo présentation",IF(K52="Message envoyé",IF(J52="","Indiquer la date d'envoi",IF(TODAY()&gt;=J52+3,"Envoyer la relance 1","Attendre la réponse")),IF(K52="Relance 1 faite",IF(TODAY()&gt;=J52+7,"Envoyer la relance 2","Attendre la réponse"),IF(K52="Relance 2 faite","Si rien sous 3 jours : Sans réponse",IF(K52="A répondu","Envoyer message 2 + vidéo workflow",IF(K52="Démo prévue","Préparer la démo avec ses produits",IF(K52="Démo faite","Envoyer l'offre et le prix",IF(K52="Client","Installer et demander un avis","Fini"))))))))</f>
+        <v>Envoyer message 1 + vidéo présentation</v>
+      </c>
+      <c r="O52" s="19"/>
+      <c r="P52" s="20" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="12" t="n">
+        <v>103</v>
+      </c>
+      <c r="B53" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C53" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D53" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="E53" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="F53" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="G53" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H53" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="I53" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="J53" s="15"/>
+      <c r="K53" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="L53" s="17" t="str">
+        <f aca="false">IF(J53="","",J53+3)</f>
+        <v/>
+      </c>
+      <c r="M53" s="17" t="str">
+        <f aca="false">IF(J53="","",J53+7)</f>
+        <v/>
+      </c>
+      <c r="N53" s="18" t="str">
+        <f aca="true">IF(K53="À contacter","Envoyer message 1 + vidéo présentation",IF(K53="Message envoyé",IF(J53="","Indiquer la date d'envoi",IF(TODAY()&gt;=J53+3,"Envoyer la relance 1","Attendre la réponse")),IF(K53="Relance 1 faite",IF(TODAY()&gt;=J53+7,"Envoyer la relance 2","Attendre la réponse"),IF(K53="Relance 2 faite","Si rien sous 3 jours : Sans réponse",IF(K53="A répondu","Envoyer message 2 + vidéo workflow",IF(K53="Démo prévue","Préparer la démo avec ses produits",IF(K53="Démo faite","Envoyer l'offre et le prix",IF(K53="Client","Installer et demander un avis","Fini"))))))))</f>
+        <v>Envoyer message 1 + vidéo présentation</v>
+      </c>
+      <c r="O53" s="19"/>
+      <c r="P53" s="20" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="12" t="n">
+        <v>101</v>
+      </c>
+      <c r="B54" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D54" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="E54" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F54" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="G54" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H54" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="I54" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="J54" s="15"/>
+      <c r="K54" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="L54" s="17" t="str">
+        <f aca="false">IF(J54="","",J54+3)</f>
+        <v/>
+      </c>
+      <c r="M54" s="17" t="str">
+        <f aca="false">IF(J54="","",J54+7)</f>
+        <v/>
+      </c>
+      <c r="N54" s="18" t="str">
+        <f aca="true">IF(K54="À contacter","Envoyer message 1 + vidéo présentation",IF(K54="Message envoyé",IF(J54="","Indiquer la date d'envoi",IF(TODAY()&gt;=J54+3,"Envoyer la relance 1","Attendre la réponse")),IF(K54="Relance 1 faite",IF(TODAY()&gt;=J54+7,"Envoyer la relance 2","Attendre la réponse"),IF(K54="Relance 2 faite","Si rien sous 3 jours : Sans réponse",IF(K54="A répondu","Envoyer message 2 + vidéo workflow",IF(K54="Démo prévue","Préparer la démo avec ses produits",IF(K54="Démo faite","Envoyer l'offre et le prix",IF(K54="Client","Installer et demander un avis","Fini"))))))))</f>
+        <v>Envoyer message 1 + vidéo présentation</v>
+      </c>
+      <c r="O54" s="19"/>
+      <c r="P54" s="20" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="12" t="n">
+        <v>105</v>
+      </c>
+      <c r="B55" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D55" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="E55" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F55" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="G55" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H55" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="I55" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="J55" s="15"/>
+      <c r="K55" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="L55" s="17" t="str">
+        <f aca="false">IF(J55="","",J55+3)</f>
+        <v/>
+      </c>
+      <c r="M55" s="17" t="str">
+        <f aca="false">IF(J55="","",J55+7)</f>
+        <v/>
+      </c>
+      <c r="N55" s="18" t="str">
+        <f aca="true">IF(K55="À contacter","Envoyer message 1 + vidéo présentation",IF(K55="Message envoyé",IF(J55="","Indiquer la date d'envoi",IF(TODAY()&gt;=J55+3,"Envoyer la relance 1","Attendre la réponse")),IF(K55="Relance 1 faite",IF(TODAY()&gt;=J55+7,"Envoyer la relance 2","Attendre la réponse"),IF(K55="Relance 2 faite","Si rien sous 3 jours : Sans réponse",IF(K55="A répondu","Envoyer message 2 + vidéo workflow",IF(K55="Démo prévue","Préparer la démo avec ses produits",IF(K55="Démo faite","Envoyer l'offre et le prix",IF(K55="Client","Installer et demander un avis","Fini"))))))))</f>
+        <v>Envoyer message 1 + vidéo présentation</v>
+      </c>
+      <c r="O55" s="19"/>
+      <c r="P55" s="20" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="12" t="n">
+        <v>102</v>
+      </c>
+      <c r="B56" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D56" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="F56" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="G56" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H56" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="I56" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="J56" s="15"/>
+      <c r="K56" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="L56" s="17" t="str">
+        <f aca="false">IF(J56="","",J56+3)</f>
+        <v/>
+      </c>
+      <c r="M56" s="17" t="str">
+        <f aca="false">IF(J56="","",J56+7)</f>
+        <v/>
+      </c>
+      <c r="N56" s="18" t="str">
+        <f aca="true">IF(K56="À contacter","Envoyer message 1 + vidéo présentation",IF(K56="Message envoyé",IF(J56="","Indiquer la date d'envoi",IF(TODAY()&gt;=J56+3,"Envoyer la relance 1","Attendre la réponse")),IF(K56="Relance 1 faite",IF(TODAY()&gt;=J56+7,"Envoyer la relance 2","Attendre la réponse"),IF(K56="Relance 2 faite","Si rien sous 3 jours : Sans réponse",IF(K56="A répondu","Envoyer message 2 + vidéo workflow",IF(K56="Démo prévue","Préparer la démo avec ses produits",IF(K56="Démo faite","Envoyer l'offre et le prix",IF(K56="Client","Installer et demander un avis","Fini"))))))))</f>
+        <v>Envoyer message 1 + vidéo présentation</v>
+      </c>
+      <c r="O56" s="19"/>
+      <c r="P56" s="20" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:P51"/>
-  <conditionalFormatting sqref="K5:K51">
+  <autoFilter ref="A4:P56"/>
+  <conditionalFormatting sqref="K5:K56">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>"Client"</formula>
     </cfRule>
@@ -3879,7 +4240,7 @@
       <formula>"Sans réponse"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C5:C51">
+  <conditionalFormatting sqref="C5:C56">
     <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>"A"</formula>
     </cfRule>
@@ -3890,17 +4251,17 @@
       <formula>"C"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N51">
+  <conditionalFormatting sqref="N5:N56">
     <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>LEFT(N5,7)="Envoyer"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" error="Choisissez un statut dans la liste." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K5:K51" type="list">
+    <dataValidation allowBlank="false" error="Choisissez un statut dans la liste." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K5:K56" type="list">
       <formula1>"À contacter,Message envoyé,Relance 1 faite,Relance 2 faite,A répondu,Démo prévue,Démo faite,Client,Pas intéressé,Sans réponse"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J51" type="date">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J56" type="date">
       <formula1>45000</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3953,6 +4314,11 @@
     <hyperlink ref="G49" r:id="rId45" display="Ouvrir WhatsApp"/>
     <hyperlink ref="G50" r:id="rId46" display="Ouvrir WhatsApp"/>
     <hyperlink ref="G51" r:id="rId47" display="Ouvrir WhatsApp"/>
+    <hyperlink ref="G52" r:id="rId48" display="Ouvrir WhatsApp"/>
+    <hyperlink ref="G53" r:id="rId49" display="Ouvrir WhatsApp"/>
+    <hyperlink ref="G54" r:id="rId50" display="Ouvrir WhatsApp"/>
+    <hyperlink ref="G55" r:id="rId51" display="Ouvrir WhatsApp"/>
+    <hyperlink ref="G56" r:id="rId52" display="Ouvrir WhatsApp"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3961,7 +4327,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId48"/>
+  <drawing r:id="rId53"/>
 </worksheet>
 </file>
 
@@ -3979,47 +4345,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>169</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="240" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>170</v>
+        <v>194</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="285" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
-        <v>172</v>
+        <v>196</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>173</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>175</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>